<commit_message>
CORRECCIONES 03 EN ARCA
</commit_message>
<xml_diff>
--- a/00000_Correcciones/Cohoorte06.xlsx
+++ b/00000_Correcciones/Cohoorte06.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\00_ENGITHUB\Modulo02_JavaScript\00000_Correcciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{211F2869-FBDD-4139-91D1-9413E8B1A88B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BCE4971-C3F7-447C-955E-1B75002496AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="92">
   <si>
     <t>Acosta Nieva, Nicole Nazarena</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>el 40% se hizo con IA</t>
+  </si>
+  <si>
+    <t>Utilizo 80% IA</t>
   </si>
 </sst>
 </file>
@@ -1851,7 +1854,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49">
         <v>1</v>
       </c>
@@ -1864,8 +1867,17 @@
       <c r="F49">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="H49">
+        <v>48</v>
+      </c>
+      <c r="I49" t="s">
+        <v>2</v>
+      </c>
+      <c r="J49">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50">
         <v>2</v>
       </c>
@@ -1879,7 +1891,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51">
         <v>3</v>
       </c>
@@ -1892,8 +1904,17 @@
       <c r="F51">
         <v>8</v>
       </c>
-    </row>
-    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="H51">
+        <v>47</v>
+      </c>
+      <c r="I51" t="s">
+        <v>2</v>
+      </c>
+      <c r="J51">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B52" s="2">
         <v>5</v>
       </c>
@@ -1914,7 +1935,7 @@
       </c>
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53">
         <v>6</v>
       </c>
@@ -1928,7 +1949,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B54" s="8">
         <v>7</v>
       </c>
@@ -1944,7 +1965,7 @@
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
     </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B55">
         <v>11</v>
       </c>
@@ -1958,7 +1979,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B56">
         <v>14</v>
       </c>
@@ -1971,8 +1992,17 @@
       <c r="F56">
         <v>8</v>
       </c>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="H56">
+        <v>49</v>
+      </c>
+      <c r="I56" t="s">
+        <v>2</v>
+      </c>
+      <c r="J56">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57">
         <v>17</v>
       </c>
@@ -1986,7 +2016,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B58">
         <v>23</v>
       </c>
@@ -2000,7 +2030,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="2">
         <v>26</v>
       </c>
@@ -2019,7 +2049,7 @@
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B60">
         <v>30</v>
       </c>
@@ -2033,7 +2063,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B61">
         <v>35</v>
       </c>
@@ -2047,7 +2077,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="62" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B62" s="3">
         <v>44</v>
       </c>
@@ -2068,7 +2098,7 @@
       </c>
       <c r="H62" s="3"/>
     </row>
-    <row r="63" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B63">
         <v>58</v>
       </c>
@@ -2082,7 +2112,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B64">
         <v>59</v>
       </c>
@@ -2096,7 +2126,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B65">
         <v>60</v>
       </c>
@@ -2109,8 +2139,20 @@
       <c r="F65">
         <v>2</v>
       </c>
-    </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H65">
+        <v>46</v>
+      </c>
+      <c r="I65" t="s">
+        <v>6</v>
+      </c>
+      <c r="J65">
+        <v>2</v>
+      </c>
+      <c r="K65" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="66" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B66">
         <v>61</v>
       </c>
@@ -2124,7 +2166,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B67">
         <v>64</v>
       </c>

</xml_diff>